<commit_message>
Fixed IT-002 and IT-003 and updated the test log with them. All tests pass now
</commit_message>
<xml_diff>
--- a/Project_Test_Log_Template.xlsx
+++ b/Project_Test_Log_Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Shubham 1\Conestoga\Semester 7\Software Safety &amp; Reliability\Group Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Shubham 1\Conestoga\Semester 7\Software Safety &amp; Reliability\Group Project\AircraftGroundControl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C99D53C-755F-4139-BA34-08E8C5CDFA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE45643-2C81-4836-A7D5-58BD8D6A23F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{E7DD175E-B3D6-47E5-B09C-23F49D44E239}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{E7DD175E-B3D6-47E5-B09C-23F49D44E239}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Definitions" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="176">
   <si>
     <t>Test ID</t>
   </si>
@@ -611,12 +611,18 @@
   <si>
     <t>#3</t>
   </si>
+  <si>
+    <t>Updated test to check logs in the executable working directory instead of repo root. Fix ensures correct file path matching where client/server actually generate logs.</t>
+  </si>
+  <si>
+    <t>Modified test to run full end-to-end scenario and validate file in runtime directory. Fix removes dependency on previous tests and ensures independent execution</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -648,13 +654,6 @@
     </font>
     <font>
       <sz val="20"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -714,7 +713,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -739,13 +738,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
@@ -1087,17 +1085,17 @@
       <c r="B1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12" t="s">
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
       <c r="J1" s="3" t="s">
         <v>10</v>
       </c>
@@ -1182,10 +1180,10 @@
       <c r="K4" t="s">
         <v>31</v>
       </c>
-      <c r="L4" s="14" t="s">
+      <c r="L4" t="s">
         <v>89</v>
       </c>
-      <c r="M4" s="14" t="s">
+      <c r="M4" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1304,7 +1302,7 @@
       <c r="I8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="14" t="s">
+      <c r="J8" t="s">
         <v>79</v>
       </c>
       <c r="K8" t="s">
@@ -1616,7 +1614,7 @@
       <c r="A21" t="s">
         <v>94</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="12" t="s">
         <v>93</v>
       </c>
       <c r="C21" s="1" t="s">
@@ -1863,7 +1861,7 @@
       <c r="H31" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J31" s="14" t="s">
+      <c r="J31" t="s">
         <v>133</v>
       </c>
       <c r="K31" t="s">
@@ -1930,7 +1928,7 @@
       <c r="H33" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J33" s="14" t="s">
+      <c r="J33" t="s">
         <v>132</v>
       </c>
       <c r="K33" t="s">
@@ -1948,7 +1946,7 @@
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="F1:I1"/>
   </mergeCells>
-  <phoneticPr fontId="6" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
@@ -1956,7 +1954,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F816C4BB-0595-4F94-9ABD-38BF074526B3}">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" customWidth="1"/>
@@ -2021,7 +2019,7 @@
       <c r="D3" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" t="s">
         <v>90</v>
       </c>
       <c r="G3" s="2" t="s">
@@ -2473,6 +2471,49 @@
       <c r="G25" t="s">
         <v>171</v>
       </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B26" t="s">
+        <v>126</v>
+      </c>
+      <c r="C26" t="s">
+        <v>168</v>
+      </c>
+      <c r="D26" t="s">
+        <v>21</v>
+      </c>
+      <c r="F26" t="s">
+        <v>91</v>
+      </c>
+      <c r="G26" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B27" t="s">
+        <v>127</v>
+      </c>
+      <c r="C27" t="s">
+        <v>168</v>
+      </c>
+      <c r="D27" t="s">
+        <v>21</v>
+      </c>
+      <c r="F27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G27" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added more system, unit and Integration tests. Added detailed comments in the test code and added DAL relevance comments in it. Updated test log and added screenshots of the passed test explorer results under documentation folder.
</commit_message>
<xml_diff>
--- a/Project_Test_Log_Template.xlsx
+++ b/Project_Test_Log_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Shubham 1\Conestoga\Semester 7\Software Safety &amp; Reliability\Group Project\AircraftGroundControl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE45643-2C81-4836-A7D5-58BD8D6A23F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEFC3334-692A-4A6D-8FC2-4440836A305B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{E7DD175E-B3D6-47E5-B09C-23F49D44E239}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{E7DD175E-B3D6-47E5-B09C-23F49D44E239}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Definitions" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="247">
   <si>
     <t>Test ID</t>
   </si>
@@ -129,9 +129,6 @@
     <t>UT-CMN-01</t>
   </si>
   <si>
-    <t>Validate Aircarft ID; Accepts Congigured ID</t>
-  </si>
-  <si>
     <t>agc::validateAircraftId()</t>
   </si>
   <si>
@@ -178,45 +175,6 @@
   </si>
   <si>
     <t>UT-CLT-008</t>
-  </si>
-  <si>
-    <t>Validate Aircraft ID; Rejects Invalid ID</t>
-  </si>
-  <si>
-    <t>Reject Oversized Payload</t>
-  </si>
-  <si>
-    <t>Reject Stale Timestamp</t>
-  </si>
-  <si>
-    <t>Telemetry Payload Round-Trip</t>
-  </si>
-  <si>
-    <t>Packet Header Population</t>
-  </si>
-  <si>
-    <t>Checksum Stability For Known Input</t>
-  </si>
-  <si>
-    <t>Generate Telemetry Sample Zero</t>
-  </si>
-  <si>
-    <t>Generate Telemetry Progression</t>
-  </si>
-  <si>
-    <t>Parse Valid Transfer Metadata</t>
-  </si>
-  <si>
-    <t>Reject Invalid Transfer Metadata</t>
-  </si>
-  <si>
-    <t>Build Transfer Status Text</t>
-  </si>
-  <si>
-    <t>Telemetry Operational Range Valid</t>
-  </si>
-  <si>
-    <t>Telemetry Operational Range Invalid</t>
   </si>
   <si>
     <t>agc::client_logic::isTelemetryWithinExpectedOperationalRange()</t>
@@ -345,9 +303,6 @@
     <t>Yinus</t>
   </si>
   <si>
-    <t>Validate Active Packet Accepts Valid Packet</t>
-  </si>
-  <si>
     <t>UT-SVR-001</t>
   </si>
   <si>
@@ -369,24 +324,6 @@
     <t>UT-SVR-007</t>
   </si>
   <si>
-    <t>Validate Active Packet Rejects Invalid Aircraft ID</t>
-  </si>
-  <si>
-    <t>Compute Total Chunks Correctly</t>
-  </si>
-  <si>
-    <t>Build Transfer Start Metadata</t>
-  </si>
-  <si>
-    <t>Trigger Command On Second Telemetry Packet</t>
-  </si>
-  <si>
-    <t>Trigger Additional Status Request On Third Telemetry Packet</t>
-  </si>
-  <si>
-    <t>Trigger Large Transfer Only Once At Fifth Telemetry Packet</t>
-  </si>
-  <si>
     <t>agc::server_logic::validateActivePacket()</t>
   </si>
   <si>
@@ -448,15 +385,6 @@
   </si>
   <si>
     <t>IT-003</t>
-  </si>
-  <si>
-    <t>End-To-End Client And Server Session Completes Successfully</t>
-  </si>
-  <si>
-    <t>Integration Logs Are Generated And Contain Expected Events</t>
-  </si>
-  <si>
-    <t>Large Transfer Produces Received File Above One Megabyte</t>
   </si>
   <si>
     <t>Logging subsystem across client and server</t>
@@ -616,6 +544,291 @@
   </si>
   <si>
     <t>Modified test to run full end-to-end scenario and validate file in runtime directory. Fix removes dependency on previous tests and ensures independent execution</t>
+  </si>
+  <si>
+    <t>ValidateAircraftId_AcceptsConfiguredId</t>
+  </si>
+  <si>
+    <t>ValidateAircraftId_RejectsUnexpectedId</t>
+  </si>
+  <si>
+    <t>ValidatePayloadSize_RejectsOversizePayload</t>
+  </si>
+  <si>
+    <t>ValidateTimestamp_RejectsPacketOutsideAllowedWindow</t>
+  </si>
+  <si>
+    <t>TelemetryPayload_RoundTripPreservesValues</t>
+  </si>
+  <si>
+    <t>MakePacket_SetsExpectedHeaderFields</t>
+  </si>
+  <si>
+    <t>ComputeChecksum_IsStableForKnownInput</t>
+  </si>
+  <si>
+    <t>GenerateTelemetry_SampleZeroMatchesExpectedValues</t>
+  </si>
+  <si>
+    <t>GenerateTelemetry_ProgressesAsSampleIndexIncreases</t>
+  </si>
+  <si>
+    <t>ParseTransferMetadata_ValidMetadataIsAccepted</t>
+  </si>
+  <si>
+    <t>ParseTransferMetadata_InvalidMetadataIsRejected</t>
+  </si>
+  <si>
+    <t>BuildTransferStatusText_ContainsAllFields</t>
+  </si>
+  <si>
+    <t>IsTelemetryWithinExpectedOperationalRange_ValidTelemetryPasses</t>
+  </si>
+  <si>
+    <t>IsTelemetryWithinExpectedOperationalRange_InvalidTelemetryFails</t>
+  </si>
+  <si>
+    <t>ValidateActivePacket_ValidPacketPasses</t>
+  </si>
+  <si>
+    <t>ValidateActivePacket_InvalidAircraftIdFails</t>
+  </si>
+  <si>
+    <t>ComputeTotalChunks_RoundsUpCorrectly</t>
+  </si>
+  <si>
+    <t>BuildTransferStartText_FormatsExpectedMetadata</t>
+  </si>
+  <si>
+    <t>ShouldSendCommand_OnlyOnTelemetryTwo</t>
+  </si>
+  <si>
+    <t>ShouldRequestAdditionalStatus_OnlyOnTelemetryThree</t>
+  </si>
+  <si>
+    <t>ShouldStartLargeTransfer_RespectsTriggerAndFlag</t>
+  </si>
+  <si>
+    <t>EndToEnd_ClientAndServerCompleteSuccessfully</t>
+  </si>
+  <si>
+    <t>Integration_LogsAreGeneratedAndContainExpectedEvents</t>
+  </si>
+  <si>
+    <t>System_LargeTransferProducesReceivedFileAboveOneMegabyte</t>
+  </si>
+  <si>
+    <t>UT-CMN-08</t>
+  </si>
+  <si>
+    <t>UT-CMN-09</t>
+  </si>
+  <si>
+    <t>TelemetryPayload_MalformedPayloadIsRejected</t>
+  </si>
+  <si>
+    <t>GenerateDiagnosticBlob_ReturnsRequestedSize</t>
+  </si>
+  <si>
+    <t>ParseTransferMetadata_MissingChecksumIsRejected</t>
+  </si>
+  <si>
+    <t>UT-CLT-009</t>
+  </si>
+  <si>
+    <t>BuildTransferStatusText_FailedTransferContainsFalseFlag</t>
+  </si>
+  <si>
+    <t>ComputeTotalChunks_ExactMultipleReturnsExactChunkCount</t>
+  </si>
+  <si>
+    <t>UT-SVR-008</t>
+  </si>
+  <si>
+    <t>UT-SVR-009</t>
+  </si>
+  <si>
+    <t>ShouldSendCommand_RemainsFalseOutsideTelemetryTwo</t>
+  </si>
+  <si>
+    <t>IT-004</t>
+  </si>
+  <si>
+    <t>IT-005</t>
+  </si>
+  <si>
+    <t>Integration_CommandAndStatusExchangeArePresentInLogs</t>
+  </si>
+  <si>
+    <t>Integration_DisconnectSequenceIsLogged</t>
+  </si>
+  <si>
+    <t>System_RuntimeArtifactsAreCreatedInOutputDirectory</t>
+  </si>
+  <si>
+    <t>System_LargeTransferMarkersAppearInCorrectOrder</t>
+  </si>
+  <si>
+    <t>Server Listening State Visibility</t>
+  </si>
+  <si>
+    <t>Transfer Completion Feedback Visibility</t>
+  </si>
+  <si>
+    <t>Connection Failure Message Clarity</t>
+  </si>
+  <si>
+    <t>ST-001</t>
+  </si>
+  <si>
+    <t>ST-002</t>
+  </si>
+  <si>
+    <t>Usability Tests (Client &amp; Server Together)</t>
+  </si>
+  <si>
+    <t>UTY-001</t>
+  </si>
+  <si>
+    <t>UTY-002</t>
+  </si>
+  <si>
+    <t>UTY-003</t>
+  </si>
+  <si>
+    <t>agc::payloadToTelemetry()</t>
+  </si>
+  <si>
+    <t>REQ-SYS-010, REQ-PKT-010</t>
+  </si>
+  <si>
+    <t>Verifies malformed telemetry payload text is rejected during deserialization.</t>
+  </si>
+  <si>
+    <t>agc::generateDiagnosticBlob()</t>
+  </si>
+  <si>
+    <t>Verifies generated large-transfer payload size matches the requested byte count.</t>
+  </si>
+  <si>
+    <t>Verifies incomplete transfer metadata is rejected by the client before file reconstruction.</t>
+  </si>
+  <si>
+    <t>Verifies failed-transfer status text includes a FALSE result and summary fields.</t>
+  </si>
+  <si>
+    <t>REQ-SYS-070, REQ-SVR-090</t>
+  </si>
+  <si>
+    <t>Verifies exact-size transfers compute the correct number of chunks without rounding error.</t>
+  </si>
+  <si>
+    <t>Verifies command dispatch logic does not trigger outside the intended telemetry count.</t>
+  </si>
+  <si>
+    <t>End-to-end runtime logs</t>
+  </si>
+  <si>
+    <t>REQ-SYS-050, REQ-SYS-080, REQ-SVR-070, REQ-SVR-080</t>
+  </si>
+  <si>
+    <t>Verifies command, command acknowledgement, data request, and status response are recorded in runtime logs.</t>
+  </si>
+  <si>
+    <t>REQ-SYS-050, REQ-CLT-090</t>
+  </si>
+  <si>
+    <t>Verifies disconnect activity is recorded by both client and server log files.</t>
+  </si>
+  <si>
+    <t>Output artifacts from full session</t>
+  </si>
+  <si>
+    <t>REQ-SYS-050, REQ-SYS-070</t>
+  </si>
+  <si>
+    <t>Verifies logs and received file are created in the executable runtime directory after a full session.</t>
+  </si>
+  <si>
+    <t>Server runtime log ordering</t>
+  </si>
+  <si>
+    <t>REQ-SYS-070, REQ-SYS-050</t>
+  </si>
+  <si>
+    <t>Verifies large-transfer start is logged before large-transfer end in the server log.</t>
+  </si>
+  <si>
+    <t>Server console UI</t>
+  </si>
+  <si>
+    <t>REQ-SYS-040, REQ-SYS-060</t>
+  </si>
+  <si>
+    <t>Verifies the operator can clearly identify that the server is in listening state before a client connects.</t>
+  </si>
+  <si>
+    <t>Client console UI</t>
+  </si>
+  <si>
+    <t>REQ-SYS-040, REQ-SYS-070</t>
+  </si>
+  <si>
+    <t>Verifies the operator can clearly identify successful large-transfer completion and generated file output.</t>
+  </si>
+  <si>
+    <t>Client console UI during failed connection</t>
+  </si>
+  <si>
+    <t>REQ-SYS-080, REQ-SYS-040</t>
+  </si>
+  <si>
+    <t>Verifies client-side error feedback is understandable when connection to the server cannot be established.</t>
+  </si>
+  <si>
+    <t>SY</t>
+  </si>
+  <si>
+    <t>UB</t>
+  </si>
+  <si>
+    <t>Malformed telemetry payload was rejected successfully by shared deserialization logic. Validation correctly prevented invalid telemetry data from being interpreted as a valid packet.</t>
+  </si>
+  <si>
+    <t>Generated diagnostic blob matched the requested payload size exactly. Large-transfer test data creation behaved as expected for 1 MB+ object generation.</t>
+  </si>
+  <si>
+    <t>Client-side metadata parser correctly rejected transfer metadata missing the checksum field. Validation ensured incomplete transfer setup information was not accepted.</t>
+  </si>
+  <si>
+    <t>Failed-transfer status text was generated correctly with TRANSFER_OK=FALSE and summary fields. Client status reporting logic handled negative completion scenarios as expected.</t>
+  </si>
+  <si>
+    <t>Chunk-count calculation returned the correct value for an exact multiple of chunk size. Server transfer logic handled boundary-size chunking without rounding error.</t>
+  </si>
+  <si>
+    <t>Command trigger logic remained false for telemetry counts outside the intended threshold. Server command-dispatch guard conditions behaved correctly for non-trigger states.</t>
+  </si>
+  <si>
+    <t>Integration logs contained the expected command, command acknowledgement, data request, and status response events. End-to-end protocol interaction was recorded correctly in runtime log files.</t>
+  </si>
+  <si>
+    <t>Disconnect sequence was logged successfully by both client and server during integration execution. Session shutdown path completed with correct traceability in runtime logs.</t>
+  </si>
+  <si>
+    <t>Runtime artifacts were generated successfully in the executable output directory. Client log, server log, and received diagnostic file were all created in the correct runtime location.</t>
+  </si>
+  <si>
+    <t>Large-transfer start and end markers appeared in the correct order in the server log. System-level transfer logging confirmed correct sequencing of major transfer events.</t>
+  </si>
+  <si>
+    <t>Server listening state was clearly visible to the operator before client connection. Console feedback provided understandable readiness status for the server application.</t>
+  </si>
+  <si>
+    <t>Large-transfer completion feedback was clear and easy for the operator to identify. Client console output communicated successful transfer completion and file generation effectively.</t>
+  </si>
+  <si>
+    <t>Connection failure message was understandable when the server was unavailable. Client-side error feedback clearly indicated the failure condition to the operator.</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1273,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC726601-BD68-44CD-B910-B47EE77E8AC0}">
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
@@ -1160,39 +1373,39 @@
         <v>28</v>
       </c>
       <c r="B4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>30</v>
       </c>
-      <c r="K4" t="s">
-        <v>31</v>
-      </c>
       <c r="L4" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="M4" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>153</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>14</v>
@@ -1207,24 +1420,24 @@
         <v>14</v>
       </c>
       <c r="J5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K5" t="s">
         <v>30</v>
       </c>
-      <c r="K5" t="s">
-        <v>31</v>
-      </c>
       <c r="L5" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="M5" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>47</v>
+        <v>154</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>14</v>
@@ -1239,24 +1452,24 @@
         <v>14</v>
       </c>
       <c r="J6" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="K6" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="L6" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="M6" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>155</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>14</v>
@@ -1271,24 +1484,24 @@
         <v>14</v>
       </c>
       <c r="J7" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="K7" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="L7" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="M7" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>156</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>14</v>
@@ -1303,24 +1516,24 @@
         <v>14</v>
       </c>
       <c r="J8" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="K8" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="L8" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="M8" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>157</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>14</v>
@@ -1335,24 +1548,24 @@
         <v>14</v>
       </c>
       <c r="J9" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="K9" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="L9" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="M9" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>158</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>14</v>
@@ -1367,24 +1580,24 @@
         <v>14</v>
       </c>
       <c r="J10" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="K10" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="L10" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="M10" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>176</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>178</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>14</v>
@@ -1395,25 +1608,28 @@
       <c r="H11" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="I11" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="J11" t="s">
-        <v>71</v>
+        <v>202</v>
       </c>
       <c r="K11" t="s">
-        <v>60</v>
+        <v>203</v>
       </c>
       <c r="L11" t="s">
-        <v>72</v>
+        <v>204</v>
       </c>
       <c r="M11" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>39</v>
+        <v>177</v>
       </c>
       <c r="B12" t="s">
-        <v>53</v>
+        <v>179</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>14</v>
@@ -1424,25 +1640,28 @@
       <c r="H12" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="I12" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="J12" t="s">
-        <v>71</v>
+        <v>205</v>
       </c>
       <c r="K12" t="s">
         <v>60</v>
       </c>
       <c r="L12" t="s">
-        <v>70</v>
+        <v>206</v>
       </c>
       <c r="M12" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B13" t="s">
-        <v>54</v>
+        <v>159</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>14</v>
@@ -1453,28 +1672,25 @@
       <c r="H13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I13" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="J13" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="K13" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="L13" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="M13" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B14" t="s">
-        <v>55</v>
+        <v>160</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>14</v>
@@ -1485,28 +1701,25 @@
       <c r="H14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I14" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="J14" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="K14" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="L14" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="M14" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>161</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>14</v>
@@ -1517,25 +1730,28 @@
       <c r="H15" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="I15" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="J15" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="K15" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="L15" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="M15" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B16" t="s">
-        <v>57</v>
+        <v>162</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>14</v>
@@ -1546,25 +1762,28 @@
       <c r="H16" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="I16" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="J16" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="K16" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L16" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="M16" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B17" t="s">
-        <v>58</v>
+        <v>163</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>14</v>
@@ -1576,46 +1795,114 @@
         <v>14</v>
       </c>
       <c r="J17" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="K17" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="L17" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="M17" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" t="s">
+        <v>164</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J18" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" s="11" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A20" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="8"/>
+      <c r="K18" t="s">
+        <v>46</v>
+      </c>
+      <c r="L18" t="s">
+        <v>48</v>
+      </c>
+      <c r="M18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" t="s">
+        <v>165</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J19" t="s">
+        <v>45</v>
+      </c>
+      <c r="K19" t="s">
+        <v>46</v>
+      </c>
+      <c r="L19" t="s">
+        <v>47</v>
+      </c>
+      <c r="M19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" t="s">
+        <v>180</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J20" t="s">
+        <v>54</v>
+      </c>
+      <c r="K20" t="s">
+        <v>50</v>
+      </c>
+      <c r="L20" t="s">
+        <v>207</v>
+      </c>
+      <c r="M20" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>94</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>93</v>
+        <v>181</v>
+      </c>
+      <c r="B21" t="s">
+        <v>182</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>14</v>
@@ -1626,92 +1913,42 @@
       <c r="H21" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I21" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="J21" t="s">
-        <v>107</v>
+        <v>49</v>
       </c>
       <c r="K21" t="s">
-        <v>108</v>
+        <v>50</v>
       </c>
       <c r="L21" t="s">
-        <v>109</v>
+        <v>208</v>
       </c>
       <c r="M21" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>95</v>
-      </c>
-      <c r="B22" t="s">
-        <v>101</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J22" t="s">
-        <v>107</v>
-      </c>
-      <c r="K22" t="s">
-        <v>108</v>
-      </c>
-      <c r="L22" t="s">
-        <v>110</v>
-      </c>
-      <c r="M22" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>96</v>
-      </c>
-      <c r="B23" t="s">
-        <v>102</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J23" t="s">
-        <v>112</v>
-      </c>
-      <c r="K23" t="s">
-        <v>67</v>
-      </c>
-      <c r="L23" t="s">
-        <v>111</v>
-      </c>
-      <c r="M23" t="s">
-        <v>92</v>
-      </c>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" s="11" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A23" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="8"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="8"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>97</v>
-      </c>
-      <c r="B24" t="s">
-        <v>103</v>
+        <v>79</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>166</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>14</v>
@@ -1726,24 +1963,24 @@
         <v>14</v>
       </c>
       <c r="J24" t="s">
-        <v>113</v>
+        <v>86</v>
       </c>
       <c r="K24" t="s">
-        <v>114</v>
+        <v>87</v>
       </c>
       <c r="L24" t="s">
-        <v>115</v>
+        <v>88</v>
       </c>
       <c r="M24" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="B25" t="s">
-        <v>104</v>
+        <v>167</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>14</v>
@@ -1754,25 +1991,28 @@
       <c r="H25" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="I25" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="J25" t="s">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="K25" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="L25" t="s">
-        <v>116</v>
+        <v>89</v>
       </c>
       <c r="M25" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="B26" t="s">
-        <v>105</v>
+        <v>168</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>14</v>
@@ -1783,76 +2023,149 @@
       <c r="H26" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="I26" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="J26" t="s">
-        <v>119</v>
+        <v>91</v>
       </c>
       <c r="K26" t="s">
-        <v>120</v>
+        <v>53</v>
       </c>
       <c r="L26" t="s">
-        <v>121</v>
+        <v>90</v>
       </c>
       <c r="M26" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>82</v>
+      </c>
+      <c r="B27" t="s">
+        <v>169</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J27" t="s">
+        <v>92</v>
+      </c>
+      <c r="K27" t="s">
+        <v>93</v>
+      </c>
+      <c r="L27" t="s">
+        <v>94</v>
+      </c>
+      <c r="M27" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>83</v>
+      </c>
+      <c r="B28" t="s">
+        <v>170</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J28" t="s">
+        <v>97</v>
+      </c>
+      <c r="K28" t="s">
+        <v>96</v>
+      </c>
+      <c r="L28" t="s">
+        <v>95</v>
+      </c>
+      <c r="M28" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>84</v>
+      </c>
+      <c r="B29" t="s">
+        <v>171</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J29" t="s">
+        <v>98</v>
+      </c>
+      <c r="K29" t="s">
+        <v>99</v>
+      </c>
+      <c r="L29" t="s">
         <v>100</v>
       </c>
-      <c r="B27" t="s">
-        <v>106</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J27" t="s">
-        <v>124</v>
-      </c>
-      <c r="K27" t="s">
-        <v>123</v>
-      </c>
-      <c r="L27" t="s">
-        <v>122</v>
-      </c>
-      <c r="M27" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" s="11" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A30" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B30" s="8"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
-      <c r="I30" s="9"/>
-      <c r="J30" s="8"/>
-      <c r="K30" s="10"/>
-      <c r="L30" s="10"/>
-      <c r="M30" s="8"/>
+      <c r="M29" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>85</v>
+      </c>
+      <c r="B30" t="s">
+        <v>172</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J30" t="s">
+        <v>103</v>
+      </c>
+      <c r="K30" t="s">
+        <v>102</v>
+      </c>
+      <c r="L30" t="s">
+        <v>101</v>
+      </c>
+      <c r="M30" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>125</v>
+        <v>184</v>
       </c>
       <c r="B31" t="s">
-        <v>128</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E31" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F31" s="1" t="s">
@@ -1861,30 +2174,30 @@
       <c r="H31" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="I31" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="J31" t="s">
-        <v>133</v>
+        <v>91</v>
       </c>
       <c r="K31" t="s">
-        <v>134</v>
+        <v>209</v>
       </c>
       <c r="L31" t="s">
-        <v>137</v>
+        <v>210</v>
       </c>
       <c r="M31" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>126</v>
+        <v>185</v>
       </c>
       <c r="B32" t="s">
-        <v>129</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E32" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>14</v>
       </c>
       <c r="F32" s="1" t="s">
@@ -1894,51 +2207,376 @@
         <v>14</v>
       </c>
       <c r="J32" t="s">
-        <v>131</v>
+        <v>97</v>
       </c>
       <c r="K32" t="s">
-        <v>135</v>
+        <v>96</v>
       </c>
       <c r="L32" t="s">
-        <v>138</v>
+        <v>211</v>
       </c>
       <c r="M32" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>127</v>
-      </c>
-      <c r="B33" t="s">
-        <v>130</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H33" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J33" t="s">
-        <v>132</v>
-      </c>
-      <c r="K33" t="s">
-        <v>136</v>
-      </c>
-      <c r="L33" t="s">
-        <v>139</v>
-      </c>
-      <c r="M33" t="s">
-        <v>90</v>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" s="11" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A34" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B34" s="8"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="10"/>
+      <c r="L34" s="10"/>
+      <c r="M34" s="8"/>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>104</v>
+      </c>
+      <c r="B35" t="s">
+        <v>173</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J35" t="s">
+        <v>109</v>
+      </c>
+      <c r="K35" t="s">
+        <v>110</v>
+      </c>
+      <c r="L35" t="s">
+        <v>113</v>
+      </c>
+      <c r="M35" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>105</v>
+      </c>
+      <c r="B36" t="s">
+        <v>174</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J36" t="s">
+        <v>107</v>
+      </c>
+      <c r="K36" t="s">
+        <v>111</v>
+      </c>
+      <c r="L36" t="s">
+        <v>114</v>
+      </c>
+      <c r="M36" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>106</v>
+      </c>
+      <c r="B37" t="s">
+        <v>175</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J37" t="s">
+        <v>108</v>
+      </c>
+      <c r="K37" t="s">
+        <v>112</v>
+      </c>
+      <c r="L37" t="s">
+        <v>115</v>
+      </c>
+      <c r="M37" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>187</v>
+      </c>
+      <c r="B38" t="s">
+        <v>189</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J38" t="s">
+        <v>212</v>
+      </c>
+      <c r="K38" t="s">
+        <v>213</v>
+      </c>
+      <c r="L38" t="s">
+        <v>214</v>
+      </c>
+      <c r="M38" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>188</v>
+      </c>
+      <c r="B39" t="s">
+        <v>190</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J39" t="s">
+        <v>212</v>
+      </c>
+      <c r="K39" t="s">
+        <v>215</v>
+      </c>
+      <c r="L39" t="s">
+        <v>216</v>
+      </c>
+      <c r="M39" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>196</v>
+      </c>
+      <c r="B40" t="s">
+        <v>191</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J40" t="s">
+        <v>217</v>
+      </c>
+      <c r="K40" t="s">
+        <v>218</v>
+      </c>
+      <c r="L40" t="s">
+        <v>219</v>
+      </c>
+      <c r="M40" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>197</v>
+      </c>
+      <c r="B41" t="s">
+        <v>192</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J41" t="s">
+        <v>220</v>
+      </c>
+      <c r="K41" t="s">
+        <v>221</v>
+      </c>
+      <c r="L41" t="s">
+        <v>222</v>
+      </c>
+      <c r="M41" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" s="11" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A43" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="B43" s="8"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="9"/>
+      <c r="I43" s="9"/>
+      <c r="J43" s="8"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="8"/>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>199</v>
+      </c>
+      <c r="B44" t="s">
+        <v>193</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J44" t="s">
+        <v>223</v>
+      </c>
+      <c r="K44" t="s">
+        <v>224</v>
+      </c>
+      <c r="L44" t="s">
+        <v>225</v>
+      </c>
+      <c r="M44" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>200</v>
+      </c>
+      <c r="B45" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H45" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J45" t="s">
+        <v>226</v>
+      </c>
+      <c r="K45" t="s">
+        <v>227</v>
+      </c>
+      <c r="L45" t="s">
+        <v>228</v>
+      </c>
+      <c r="M45" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>201</v>
+      </c>
+      <c r="B46" t="s">
+        <v>195</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J46" t="s">
+        <v>229</v>
+      </c>
+      <c r="K46" t="s">
+        <v>230</v>
+      </c>
+      <c r="L46" t="s">
+        <v>231</v>
+      </c>
+      <c r="M46" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1954,7 +2592,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F816C4BB-0595-4F94-9ABD-38BF074526B3}">
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" customWidth="1"/>
@@ -1991,7 +2629,7 @@
         <v>46123</v>
       </c>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>116</v>
       </c>
       <c r="C2" t="s">
         <v>23</v>
@@ -2000,10 +2638,10 @@
         <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>141</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -2011,7 +2649,7 @@
         <v>46123</v>
       </c>
       <c r="B3" t="s">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="C3" t="s">
         <v>23</v>
@@ -2020,10 +2658,10 @@
         <v>21</v>
       </c>
       <c r="F3" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>143</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -2031,7 +2669,7 @@
         <v>46123</v>
       </c>
       <c r="B4" t="s">
-        <v>144</v>
+        <v>120</v>
       </c>
       <c r="C4" t="s">
         <v>23</v>
@@ -2040,10 +2678,10 @@
         <v>21</v>
       </c>
       <c r="F4" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="G4" t="s">
-        <v>145</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -2051,7 +2689,7 @@
         <v>46123</v>
       </c>
       <c r="B5" t="s">
-        <v>146</v>
+        <v>122</v>
       </c>
       <c r="C5" t="s">
         <v>23</v>
@@ -2060,10 +2698,10 @@
         <v>21</v>
       </c>
       <c r="F5" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="G5" t="s">
-        <v>147</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -2071,7 +2709,7 @@
         <v>46123</v>
       </c>
       <c r="B6" t="s">
-        <v>148</v>
+        <v>124</v>
       </c>
       <c r="C6" t="s">
         <v>23</v>
@@ -2080,10 +2718,10 @@
         <v>21</v>
       </c>
       <c r="F6" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="G6" t="s">
-        <v>149</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -2091,7 +2729,7 @@
         <v>46123</v>
       </c>
       <c r="B7" t="s">
-        <v>150</v>
+        <v>126</v>
       </c>
       <c r="C7" t="s">
         <v>23</v>
@@ -2100,10 +2738,10 @@
         <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="G7" t="s">
-        <v>151</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -2111,7 +2749,7 @@
         <v>46123</v>
       </c>
       <c r="B8" t="s">
-        <v>152</v>
+        <v>128</v>
       </c>
       <c r="C8" t="s">
         <v>23</v>
@@ -2120,10 +2758,10 @@
         <v>21</v>
       </c>
       <c r="F8" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="G8" t="s">
-        <v>153</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -2131,7 +2769,7 @@
         <v>46123</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
         <v>23</v>
@@ -2140,10 +2778,10 @@
         <v>21</v>
       </c>
       <c r="F9" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="G9" t="s">
-        <v>154</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -2151,7 +2789,7 @@
         <v>46123</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
         <v>23</v>
@@ -2160,10 +2798,10 @@
         <v>21</v>
       </c>
       <c r="F10" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="G10" t="s">
-        <v>155</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -2171,7 +2809,7 @@
         <v>46123</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
         <v>23</v>
@@ -2180,10 +2818,10 @@
         <v>21</v>
       </c>
       <c r="F11" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="G11" t="s">
-        <v>156</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -2191,7 +2829,7 @@
         <v>46123</v>
       </c>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
         <v>23</v>
@@ -2200,10 +2838,10 @@
         <v>21</v>
       </c>
       <c r="F12" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="G12" t="s">
-        <v>157</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -2211,7 +2849,7 @@
         <v>46123</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
         <v>23</v>
@@ -2220,10 +2858,10 @@
         <v>21</v>
       </c>
       <c r="F13" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="G13" t="s">
-        <v>158</v>
+        <v>134</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -2231,7 +2869,7 @@
         <v>46123</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
         <v>23</v>
@@ -2240,10 +2878,10 @@
         <v>21</v>
       </c>
       <c r="F14" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="G14" t="s">
-        <v>159</v>
+        <v>135</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -2251,7 +2889,7 @@
         <v>46123</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15" t="s">
         <v>23</v>
@@ -2260,10 +2898,10 @@
         <v>21</v>
       </c>
       <c r="F15" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="G15" t="s">
-        <v>160</v>
+        <v>136</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -2271,7 +2909,7 @@
         <v>46123</v>
       </c>
       <c r="B16" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="C16" t="s">
         <v>23</v>
@@ -2280,10 +2918,10 @@
         <v>21</v>
       </c>
       <c r="F16" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="G16" t="s">
-        <v>161</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2291,7 +2929,7 @@
         <v>46123</v>
       </c>
       <c r="B17" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="C17" t="s">
         <v>23</v>
@@ -2300,10 +2938,10 @@
         <v>21</v>
       </c>
       <c r="F17" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="G17" t="s">
-        <v>162</v>
+        <v>138</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -2311,7 +2949,7 @@
         <v>46123</v>
       </c>
       <c r="B18" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="C18" t="s">
         <v>23</v>
@@ -2320,10 +2958,10 @@
         <v>21</v>
       </c>
       <c r="F18" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="G18" t="s">
-        <v>163</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -2331,7 +2969,7 @@
         <v>46123</v>
       </c>
       <c r="B19" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="C19" t="s">
         <v>23</v>
@@ -2340,10 +2978,10 @@
         <v>21</v>
       </c>
       <c r="F19" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="G19" t="s">
-        <v>164</v>
+        <v>140</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -2351,7 +2989,7 @@
         <v>46123</v>
       </c>
       <c r="B20" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="C20" t="s">
         <v>23</v>
@@ -2360,10 +2998,10 @@
         <v>21</v>
       </c>
       <c r="F20" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="G20" t="s">
-        <v>165</v>
+        <v>141</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -2371,7 +3009,7 @@
         <v>46123</v>
       </c>
       <c r="B21" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="C21" t="s">
         <v>23</v>
@@ -2380,10 +3018,10 @@
         <v>21</v>
       </c>
       <c r="F21" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="G21" t="s">
-        <v>166</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -2391,7 +3029,7 @@
         <v>46123</v>
       </c>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="C22" t="s">
         <v>23</v>
@@ -2400,10 +3038,10 @@
         <v>21</v>
       </c>
       <c r="F22" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="G22" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -2411,19 +3049,19 @@
         <v>46123</v>
       </c>
       <c r="B23" t="s">
-        <v>125</v>
+        <v>104</v>
       </c>
       <c r="C23" t="s">
-        <v>168</v>
+        <v>144</v>
       </c>
       <c r="D23" t="s">
         <v>21</v>
       </c>
       <c r="F23" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="G23" t="s">
-        <v>169</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -2431,22 +3069,22 @@
         <v>46123</v>
       </c>
       <c r="B24" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="C24" t="s">
-        <v>168</v>
+        <v>144</v>
       </c>
       <c r="D24" t="s">
         <v>20</v>
       </c>
       <c r="E24" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="F24" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="G24" t="s">
-        <v>170</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -2454,22 +3092,22 @@
         <v>46123</v>
       </c>
       <c r="B25" t="s">
-        <v>127</v>
+        <v>106</v>
       </c>
       <c r="C25" t="s">
-        <v>168</v>
+        <v>144</v>
       </c>
       <c r="D25" t="s">
         <v>20</v>
       </c>
       <c r="E25" t="s">
-        <v>173</v>
+        <v>149</v>
       </c>
       <c r="F25" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="G25" t="s">
-        <v>171</v>
+        <v>147</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -2477,19 +3115,19 @@
         <v>46126</v>
       </c>
       <c r="B26" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="C26" t="s">
-        <v>168</v>
+        <v>144</v>
       </c>
       <c r="D26" t="s">
         <v>21</v>
       </c>
       <c r="F26" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="G26" t="s">
-        <v>174</v>
+        <v>150</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -2497,23 +3135,760 @@
         <v>46126</v>
       </c>
       <c r="B27" t="s">
+        <v>106</v>
+      </c>
+      <c r="C27" t="s">
+        <v>144</v>
+      </c>
+      <c r="D27" t="s">
+        <v>21</v>
+      </c>
+      <c r="F27" t="s">
+        <v>76</v>
+      </c>
+      <c r="G27" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B28" t="s">
+        <v>116</v>
+      </c>
+      <c r="C28" t="s">
+        <v>23</v>
+      </c>
+      <c r="D28" t="s">
+        <v>21</v>
+      </c>
+      <c r="F28" t="s">
+        <v>76</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B29" t="s">
+        <v>118</v>
+      </c>
+      <c r="C29" t="s">
+        <v>23</v>
+      </c>
+      <c r="D29" t="s">
+        <v>21</v>
+      </c>
+      <c r="F29" t="s">
+        <v>76</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B30" t="s">
+        <v>120</v>
+      </c>
+      <c r="C30" t="s">
+        <v>23</v>
+      </c>
+      <c r="D30" t="s">
+        <v>21</v>
+      </c>
+      <c r="F30" t="s">
+        <v>76</v>
+      </c>
+      <c r="G30" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B31" t="s">
+        <v>122</v>
+      </c>
+      <c r="C31" t="s">
+        <v>23</v>
+      </c>
+      <c r="D31" t="s">
+        <v>21</v>
+      </c>
+      <c r="F31" t="s">
+        <v>78</v>
+      </c>
+      <c r="G31" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B32" t="s">
+        <v>124</v>
+      </c>
+      <c r="C32" t="s">
+        <v>23</v>
+      </c>
+      <c r="D32" t="s">
+        <v>21</v>
+      </c>
+      <c r="F32" t="s">
+        <v>77</v>
+      </c>
+      <c r="G32" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B33" t="s">
+        <v>126</v>
+      </c>
+      <c r="C33" t="s">
+        <v>23</v>
+      </c>
+      <c r="D33" t="s">
+        <v>21</v>
+      </c>
+      <c r="F33" t="s">
+        <v>76</v>
+      </c>
+      <c r="G33" t="s">
         <v>127</v>
       </c>
-      <c r="C27" t="s">
-        <v>168</v>
-      </c>
-      <c r="D27" t="s">
-        <v>21</v>
-      </c>
-      <c r="F27" t="s">
-        <v>90</v>
-      </c>
-      <c r="G27" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G28"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B34" t="s">
+        <v>128</v>
+      </c>
+      <c r="C34" t="s">
+        <v>23</v>
+      </c>
+      <c r="D34" t="s">
+        <v>21</v>
+      </c>
+      <c r="F34" t="s">
+        <v>76</v>
+      </c>
+      <c r="G34" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B35" t="s">
+        <v>37</v>
+      </c>
+      <c r="C35" t="s">
+        <v>23</v>
+      </c>
+      <c r="D35" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35" t="s">
+        <v>77</v>
+      </c>
+      <c r="G35" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B36" t="s">
+        <v>38</v>
+      </c>
+      <c r="C36" t="s">
+        <v>23</v>
+      </c>
+      <c r="D36" t="s">
+        <v>21</v>
+      </c>
+      <c r="F36" t="s">
+        <v>78</v>
+      </c>
+      <c r="G36" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B37" t="s">
+        <v>39</v>
+      </c>
+      <c r="C37" t="s">
+        <v>23</v>
+      </c>
+      <c r="D37" t="s">
+        <v>21</v>
+      </c>
+      <c r="F37" t="s">
+        <v>78</v>
+      </c>
+      <c r="G37" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B38" t="s">
+        <v>40</v>
+      </c>
+      <c r="C38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D38" t="s">
+        <v>21</v>
+      </c>
+      <c r="F38" t="s">
+        <v>77</v>
+      </c>
+      <c r="G38" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B39" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" t="s">
+        <v>23</v>
+      </c>
+      <c r="D39" t="s">
+        <v>21</v>
+      </c>
+      <c r="F39" t="s">
+        <v>77</v>
+      </c>
+      <c r="G39" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B40" t="s">
+        <v>42</v>
+      </c>
+      <c r="C40" t="s">
+        <v>23</v>
+      </c>
+      <c r="D40" t="s">
+        <v>21</v>
+      </c>
+      <c r="F40" t="s">
+        <v>76</v>
+      </c>
+      <c r="G40" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B41" t="s">
+        <v>43</v>
+      </c>
+      <c r="C41" t="s">
+        <v>23</v>
+      </c>
+      <c r="D41" t="s">
+        <v>21</v>
+      </c>
+      <c r="F41" t="s">
+        <v>76</v>
+      </c>
+      <c r="G41" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B42" t="s">
+        <v>79</v>
+      </c>
+      <c r="C42" t="s">
+        <v>23</v>
+      </c>
+      <c r="D42" t="s">
+        <v>21</v>
+      </c>
+      <c r="F42" t="s">
+        <v>76</v>
+      </c>
+      <c r="G42" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B43" t="s">
+        <v>80</v>
+      </c>
+      <c r="C43" t="s">
+        <v>23</v>
+      </c>
+      <c r="D43" t="s">
+        <v>21</v>
+      </c>
+      <c r="F43" t="s">
+        <v>76</v>
+      </c>
+      <c r="G43" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B44" t="s">
+        <v>81</v>
+      </c>
+      <c r="C44" t="s">
+        <v>23</v>
+      </c>
+      <c r="D44" t="s">
+        <v>21</v>
+      </c>
+      <c r="F44" t="s">
+        <v>78</v>
+      </c>
+      <c r="G44" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B45" t="s">
+        <v>82</v>
+      </c>
+      <c r="C45" t="s">
+        <v>23</v>
+      </c>
+      <c r="D45" t="s">
+        <v>21</v>
+      </c>
+      <c r="F45" t="s">
+        <v>77</v>
+      </c>
+      <c r="G45" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B46" t="s">
+        <v>83</v>
+      </c>
+      <c r="C46" t="s">
+        <v>23</v>
+      </c>
+      <c r="D46" t="s">
+        <v>21</v>
+      </c>
+      <c r="F46" t="s">
+        <v>77</v>
+      </c>
+      <c r="G46" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B47" t="s">
+        <v>84</v>
+      </c>
+      <c r="C47" t="s">
+        <v>23</v>
+      </c>
+      <c r="D47" t="s">
+        <v>21</v>
+      </c>
+      <c r="F47" t="s">
+        <v>78</v>
+      </c>
+      <c r="G47" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B48" t="s">
+        <v>85</v>
+      </c>
+      <c r="C48" t="s">
+        <v>23</v>
+      </c>
+      <c r="D48" t="s">
+        <v>21</v>
+      </c>
+      <c r="F48" t="s">
+        <v>77</v>
+      </c>
+      <c r="G48" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B49" t="s">
+        <v>104</v>
+      </c>
+      <c r="C49" t="s">
+        <v>144</v>
+      </c>
+      <c r="D49" t="s">
+        <v>21</v>
+      </c>
+      <c r="F49" t="s">
+        <v>78</v>
+      </c>
+      <c r="G49" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B50" t="s">
+        <v>105</v>
+      </c>
+      <c r="C50" t="s">
+        <v>144</v>
+      </c>
+      <c r="D50" t="s">
+        <v>21</v>
+      </c>
+      <c r="F50" t="s">
+        <v>77</v>
+      </c>
+      <c r="G50" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B51" t="s">
+        <v>106</v>
+      </c>
+      <c r="C51" t="s">
+        <v>144</v>
+      </c>
+      <c r="D51" t="s">
+        <v>21</v>
+      </c>
+      <c r="F51" t="s">
+        <v>76</v>
+      </c>
+      <c r="G51" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B52" t="s">
+        <v>176</v>
+      </c>
+      <c r="C52" t="s">
+        <v>23</v>
+      </c>
+      <c r="D52" t="s">
+        <v>21</v>
+      </c>
+      <c r="F52" t="s">
+        <v>78</v>
+      </c>
+      <c r="G52" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B53" t="s">
+        <v>177</v>
+      </c>
+      <c r="C53" t="s">
+        <v>23</v>
+      </c>
+      <c r="D53" t="s">
+        <v>21</v>
+      </c>
+      <c r="F53" t="s">
+        <v>77</v>
+      </c>
+      <c r="G53" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B54" t="s">
+        <v>44</v>
+      </c>
+      <c r="C54" t="s">
+        <v>23</v>
+      </c>
+      <c r="D54" t="s">
+        <v>21</v>
+      </c>
+      <c r="F54" t="s">
+        <v>78</v>
+      </c>
+      <c r="G54" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B55" t="s">
+        <v>181</v>
+      </c>
+      <c r="C55" t="s">
+        <v>23</v>
+      </c>
+      <c r="D55" t="s">
+        <v>21</v>
+      </c>
+      <c r="F55" t="s">
+        <v>76</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B56" t="s">
+        <v>184</v>
+      </c>
+      <c r="C56" t="s">
+        <v>23</v>
+      </c>
+      <c r="D56" t="s">
+        <v>21</v>
+      </c>
+      <c r="F56" t="s">
+        <v>76</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B57" t="s">
+        <v>185</v>
+      </c>
+      <c r="C57" t="s">
+        <v>23</v>
+      </c>
+      <c r="D57" t="s">
+        <v>21</v>
+      </c>
+      <c r="F57" t="s">
+        <v>78</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A58" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B58" t="s">
+        <v>187</v>
+      </c>
+      <c r="C58" t="s">
+        <v>144</v>
+      </c>
+      <c r="D58" t="s">
+        <v>21</v>
+      </c>
+      <c r="F58" t="s">
+        <v>76</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B59" t="s">
+        <v>188</v>
+      </c>
+      <c r="C59" t="s">
+        <v>144</v>
+      </c>
+      <c r="D59" t="s">
+        <v>21</v>
+      </c>
+      <c r="F59" t="s">
+        <v>76</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B60" t="s">
+        <v>196</v>
+      </c>
+      <c r="C60" t="s">
+        <v>232</v>
+      </c>
+      <c r="D60" t="s">
+        <v>21</v>
+      </c>
+      <c r="F60" t="s">
+        <v>78</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B61" t="s">
+        <v>197</v>
+      </c>
+      <c r="C61" t="s">
+        <v>232</v>
+      </c>
+      <c r="D61" t="s">
+        <v>21</v>
+      </c>
+      <c r="F61" t="s">
+        <v>77</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B62" t="s">
+        <v>199</v>
+      </c>
+      <c r="C62" t="s">
+        <v>233</v>
+      </c>
+      <c r="D62" t="s">
+        <v>21</v>
+      </c>
+      <c r="F62" t="s">
+        <v>77</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B63" t="s">
+        <v>200</v>
+      </c>
+      <c r="C63" t="s">
+        <v>233</v>
+      </c>
+      <c r="D63" t="s">
+        <v>21</v>
+      </c>
+      <c r="F63" t="s">
+        <v>76</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" s="7">
+        <v>46126</v>
+      </c>
+      <c r="B64" t="s">
+        <v>201</v>
+      </c>
+      <c r="C64" t="s">
+        <v>233</v>
+      </c>
+      <c r="D64" t="s">
+        <v>21</v>
+      </c>
+      <c r="F64" t="s">
+        <v>78</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>246</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>